<commit_message>
Bulk filing: repeated sections by _2 suffix; tidier column matching
- Sheet and API carry every repeating section the PRD allows:
  complainants (from 2), accused, accused addresses and persons
  responsible (_1_2 nested), cheques, notices, witnesses and other
  pending cases. The extra sheets are gone; repeats are _2, _3 columns.
- Fields the sheet lacked are added: witnesses, persons responsible'
  contacts and address, JUR-5, PRY-1, further complainants.
- Intake builds every complainant with its own documents; scrutiny
  checks every complainant and witness.
- Column matching: required fields first with a count, repeated
  sections on tabs, optional fields behind a toggle, and the two
  sides marked with the ON Courts and Excel icons.
- Demo files use _2 columns, witnesses and a second accused.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/demo-files/tata-capital-recovery-mis.xlsx
+++ b/demo-files/tata-capital-recovery-mis.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="353" uniqueCount="205">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="216">
   <si>
     <t>Sr No</t>
   </si>
@@ -100,6 +100,30 @@
     <t>Recovered After Notice</t>
   </si>
   <si>
+    <t>Chq No_2</t>
+  </si>
+  <si>
+    <t>Chq Dt_2</t>
+  </si>
+  <si>
+    <t>Chq Amount (Rs)_2</t>
+  </si>
+  <si>
+    <t>Drawee Bank IFSC_2</t>
+  </si>
+  <si>
+    <t>Drawer A/c No_2</t>
+  </si>
+  <si>
+    <t>Presented On_2</t>
+  </si>
+  <si>
+    <t>Bounce Date_2</t>
+  </si>
+  <si>
+    <t>Bounce Reason_2</t>
+  </si>
+  <si>
     <t>TCL-AHD-PL-1001</t>
   </si>
   <si>
@@ -445,6 +469,9 @@
     <t>9, Sahjanand Park, Paldi</t>
   </si>
   <si>
+    <t>VADODARA</t>
+  </si>
+  <si>
     <t>380006</t>
   </si>
   <si>
@@ -526,16 +553,22 @@
     <t>RG25366011IN</t>
   </si>
   <si>
+    <t>253661</t>
+  </si>
+  <si>
+    <t>1,20,000</t>
+  </si>
+  <si>
     <t>TCL-AHD-PL-1010</t>
   </si>
   <si>
-    <t>Rupal H. Chauhan</t>
+    <t>Shree Ganesh Traders</t>
   </si>
   <si>
     <t>+91 98790 12310</t>
   </si>
   <si>
-    <t>rupal.chauhan@mail.example</t>
+    <t>ganesh.traders@mail.example</t>
   </si>
   <si>
     <t>18, Nilkanth Society, Navrangpura</t>
@@ -1008,7 +1041,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:AC13"/>
+  <dimension ref="A1:AK13"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
@@ -1034,9 +1067,16 @@
     <col min="26" max="26" width="15" customWidth="1"/>
     <col min="27" max="28" width="14" customWidth="1"/>
     <col min="29" max="29" width="26" customWidth="1"/>
+    <col min="30" max="31" width="14" customWidth="1"/>
+    <col min="32" max="32" width="21" customWidth="1"/>
+    <col min="33" max="33" width="22" customWidth="1"/>
+    <col min="34" max="34" width="19" customWidth="1"/>
+    <col min="35" max="35" width="18" customWidth="1"/>
+    <col min="36" max="36" width="17" customWidth="1"/>
+    <col min="37" max="37" width="19" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:29" s="1" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:37" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1123,6 +1163,30 @@
       </c>
       <c r="AC1" s="1" t="s">
         <v>28</v>
+      </c>
+      <c r="AD1" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="AH1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="AI1" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="AJ1" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="AK1" s="1" t="s">
+        <v>36</v>
       </c>
     </row>
     <row r="2" spans="1:29" x14ac:dyDescent="0.25">
@@ -1130,85 +1194,85 @@
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>29</v>
+        <v>37</v>
       </c>
       <c r="C2" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D2" t="s">
-        <v>31</v>
+        <v>39</v>
       </c>
       <c r="E2" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G2" t="s">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="H2" t="s">
-        <v>35</v>
+        <v>43</v>
       </c>
       <c r="I2" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="J2" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K2" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="L2" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="M2" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="N2" t="s">
-        <v>41</v>
+        <v>49</v>
       </c>
       <c r="O2" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="P2" t="s">
-        <v>43</v>
+        <v>51</v>
       </c>
       <c r="Q2" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="R2" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="S2" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T2" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U2" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="V2" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W2" t="s">
-        <v>50</v>
+        <v>58</v>
       </c>
       <c r="X2" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y2" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="Z2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA2" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB2" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC2">
         <v>0</v>
@@ -1219,85 +1283,85 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
+        <v>62</v>
+      </c>
+      <c r="C3" t="s">
+        <v>38</v>
+      </c>
+      <c r="D3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E3" t="s">
+        <v>40</v>
+      </c>
+      <c r="F3" t="s">
+        <v>41</v>
+      </c>
+      <c r="G3" t="s">
+        <v>64</v>
+      </c>
+      <c r="H3" t="s">
+        <v>65</v>
+      </c>
+      <c r="I3" t="s">
+        <v>66</v>
+      </c>
+      <c r="J3" t="s">
+        <v>45</v>
+      </c>
+      <c r="K3" t="s">
+        <v>67</v>
+      </c>
+      <c r="L3" t="s">
+        <v>68</v>
+      </c>
+      <c r="M3" t="s">
+        <v>69</v>
+      </c>
+      <c r="N3" t="s">
+        <v>70</v>
+      </c>
+      <c r="O3" t="s">
+        <v>71</v>
+      </c>
+      <c r="P3" t="s">
+        <v>72</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>73</v>
+      </c>
+      <c r="R3" t="s">
+        <v>74</v>
+      </c>
+      <c r="S3" t="s">
         <v>54</v>
       </c>
-      <c r="C3" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" t="s">
+      <c r="T3" t="s">
         <v>55</v>
       </c>
-      <c r="E3" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H3" t="s">
+      <c r="U3" t="s">
+        <v>75</v>
+      </c>
+      <c r="V3" t="s">
         <v>57</v>
       </c>
-      <c r="I3" t="s">
-        <v>58</v>
-      </c>
-      <c r="J3" t="s">
-        <v>37</v>
-      </c>
-      <c r="K3" t="s">
+      <c r="W3" t="s">
+        <v>76</v>
+      </c>
+      <c r="X3" t="s">
         <v>59</v>
       </c>
-      <c r="L3" t="s">
-        <v>60</v>
-      </c>
-      <c r="M3" t="s">
+      <c r="Y3" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA3" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB3" t="s">
         <v>61</v>
-      </c>
-      <c r="N3" t="s">
-        <v>62</v>
-      </c>
-      <c r="O3" t="s">
-        <v>63</v>
-      </c>
-      <c r="P3" t="s">
-        <v>64</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>65</v>
-      </c>
-      <c r="R3" t="s">
-        <v>66</v>
-      </c>
-      <c r="S3" t="s">
-        <v>46</v>
-      </c>
-      <c r="T3" t="s">
-        <v>47</v>
-      </c>
-      <c r="U3" t="s">
-        <v>67</v>
-      </c>
-      <c r="V3" t="s">
-        <v>49</v>
-      </c>
-      <c r="W3" t="s">
-        <v>68</v>
-      </c>
-      <c r="X3" t="s">
-        <v>51</v>
-      </c>
-      <c r="Y3" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z3" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA3" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB3" t="s">
-        <v>53</v>
       </c>
       <c r="AC3">
         <v>0</v>
@@ -1308,85 +1372,85 @@
         <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="C4" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D4" t="s">
-        <v>72</v>
+        <v>80</v>
       </c>
       <c r="E4" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>81</v>
       </c>
       <c r="H4" t="s">
-        <v>74</v>
+        <v>82</v>
       </c>
       <c r="I4" t="s">
-        <v>75</v>
+        <v>83</v>
       </c>
       <c r="J4" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K4" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="L4" t="s">
-        <v>77</v>
+        <v>85</v>
       </c>
       <c r="M4" t="s">
-        <v>78</v>
+        <v>86</v>
       </c>
       <c r="N4" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="O4" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="P4" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="Q4" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="R4" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="S4" t="s">
-        <v>84</v>
+        <v>92</v>
       </c>
       <c r="T4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U4" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="V4" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="W4" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="X4" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y4" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="Z4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA4" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB4" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC4">
         <v>0</v>
@@ -1397,85 +1461,85 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>89</v>
+        <v>97</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D5" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="E5" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G5" t="s">
+        <v>99</v>
+      </c>
+      <c r="H5" t="s">
+        <v>100</v>
+      </c>
+      <c r="I5" t="s">
+        <v>101</v>
+      </c>
+      <c r="J5" t="s">
+        <v>45</v>
+      </c>
+      <c r="K5" t="s">
+        <v>102</v>
+      </c>
+      <c r="L5" t="s">
+        <v>103</v>
+      </c>
+      <c r="M5" t="s">
+        <v>104</v>
+      </c>
+      <c r="N5" t="s">
+        <v>105</v>
+      </c>
+      <c r="O5" t="s">
+        <v>106</v>
+      </c>
+      <c r="P5" t="s">
+        <v>107</v>
+      </c>
+      <c r="Q5" t="s">
         <v>91</v>
       </c>
-      <c r="H5" t="s">
-        <v>92</v>
-      </c>
-      <c r="I5" t="s">
-        <v>93</v>
-      </c>
-      <c r="J5" t="s">
-        <v>37</v>
-      </c>
-      <c r="K5" t="s">
-        <v>94</v>
-      </c>
-      <c r="L5" t="s">
-        <v>95</v>
-      </c>
-      <c r="M5" t="s">
-        <v>96</v>
-      </c>
-      <c r="N5" t="s">
-        <v>97</v>
-      </c>
-      <c r="O5" t="s">
-        <v>98</v>
-      </c>
-      <c r="P5" t="s">
-        <v>99</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>83</v>
-      </c>
       <c r="R5" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="S5" t="s">
-        <v>101</v>
+        <v>109</v>
       </c>
       <c r="T5" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U5" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="V5" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W5" t="s">
-        <v>103</v>
+        <v>111</v>
       </c>
       <c r="X5" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y5" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="Z5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA5" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB5" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC5">
         <v>0</v>
@@ -1486,85 +1550,85 @@
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>105</v>
+        <v>113</v>
       </c>
       <c r="C6" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="D6" t="s">
-        <v>107</v>
+        <v>115</v>
       </c>
       <c r="E6" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G6" t="s">
-        <v>108</v>
+        <v>116</v>
       </c>
       <c r="H6" t="s">
-        <v>109</v>
+        <v>117</v>
       </c>
       <c r="I6" t="s">
-        <v>110</v>
+        <v>118</v>
       </c>
       <c r="J6" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K6" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L6" t="s">
-        <v>112</v>
+        <v>120</v>
       </c>
       <c r="M6" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="N6" t="s">
-        <v>114</v>
+        <v>122</v>
       </c>
       <c r="O6" t="s">
-        <v>115</v>
+        <v>123</v>
       </c>
       <c r="P6" t="s">
-        <v>116</v>
+        <v>124</v>
       </c>
       <c r="Q6" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="R6" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="S6" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T6" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U6" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="V6" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W6" t="s">
-        <v>119</v>
+        <v>127</v>
       </c>
       <c r="X6" t="s">
-        <v>120</v>
+        <v>128</v>
       </c>
       <c r="Y6" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="Z6" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="AA6" t="s">
-        <v>122</v>
+        <v>130</v>
       </c>
       <c r="AB6" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC6">
         <v>0</v>
@@ -1575,85 +1639,85 @@
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>123</v>
+        <v>131</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>124</v>
+        <v>132</v>
       </c>
       <c r="E7" t="s">
-        <v>125</v>
+        <v>133</v>
       </c>
       <c r="F7" t="s">
-        <v>126</v>
+        <v>134</v>
       </c>
       <c r="G7" t="s">
-        <v>127</v>
+        <v>135</v>
       </c>
       <c r="H7" t="s">
-        <v>128</v>
+        <v>136</v>
       </c>
       <c r="I7" t="s">
-        <v>129</v>
+        <v>137</v>
       </c>
       <c r="J7" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K7" t="s">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="L7" t="s">
-        <v>130</v>
+        <v>138</v>
       </c>
       <c r="M7" t="s">
-        <v>131</v>
+        <v>139</v>
       </c>
       <c r="N7" t="s">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="O7" t="s">
-        <v>133</v>
+        <v>141</v>
       </c>
       <c r="P7" t="s">
-        <v>134</v>
+        <v>142</v>
       </c>
       <c r="Q7" t="s">
-        <v>66</v>
+        <v>74</v>
       </c>
       <c r="R7" t="s">
-        <v>135</v>
+        <v>143</v>
       </c>
       <c r="S7" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T7" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U7" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="V7" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="W7" t="s">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="X7" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y7" t="s">
-        <v>138</v>
+        <v>146</v>
       </c>
       <c r="Z7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA7" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB7" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC7">
         <v>0</v>
@@ -1664,85 +1728,85 @@
         <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>139</v>
+        <v>147</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D8" t="s">
-        <v>140</v>
+        <v>148</v>
       </c>
       <c r="E8" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s">
-        <v>141</v>
+        <v>149</v>
       </c>
       <c r="H8" t="s">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="I8" t="s">
-        <v>143</v>
+        <v>151</v>
       </c>
       <c r="J8" t="s">
-        <v>37</v>
+        <v>152</v>
       </c>
       <c r="K8" t="s">
-        <v>144</v>
+        <v>153</v>
       </c>
       <c r="L8" t="s">
-        <v>145</v>
+        <v>154</v>
       </c>
       <c r="M8" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="N8" t="s">
-        <v>146</v>
+        <v>155</v>
       </c>
       <c r="O8" t="s">
-        <v>147</v>
+        <v>156</v>
       </c>
       <c r="P8" t="s">
-        <v>148</v>
+        <v>157</v>
       </c>
       <c r="Q8" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="R8" t="s">
-        <v>45</v>
+        <v>53</v>
       </c>
       <c r="S8" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T8" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U8" t="s">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="V8" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W8" t="s">
-        <v>149</v>
+        <v>158</v>
       </c>
       <c r="X8" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y8" t="s">
-        <v>52</v>
+        <v>60</v>
       </c>
       <c r="Z8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA8" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB8" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC8">
         <v>25000</v>
@@ -1753,177 +1817,201 @@
         <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>150</v>
+        <v>159</v>
       </c>
       <c r="C9" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D9" t="s">
-        <v>151</v>
+        <v>160</v>
       </c>
       <c r="E9" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F9" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G9" t="s">
-        <v>152</v>
+        <v>161</v>
       </c>
       <c r="H9" t="s">
-        <v>153</v>
+        <v>162</v>
       </c>
       <c r="I9" t="s">
-        <v>154</v>
+        <v>163</v>
       </c>
       <c r="J9" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="L9" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="M9" t="s">
+        <v>69</v>
+      </c>
+      <c r="N9" t="s">
+        <v>166</v>
+      </c>
+      <c r="O9" t="s">
+        <v>167</v>
+      </c>
+      <c r="P9" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q9" t="s">
+        <v>73</v>
+      </c>
+      <c r="R9" t="s">
+        <v>74</v>
+      </c>
+      <c r="S9" t="s">
+        <v>54</v>
+      </c>
+      <c r="T9" t="s">
+        <v>55</v>
+      </c>
+      <c r="U9" t="s">
+        <v>75</v>
+      </c>
+      <c r="V9" t="s">
+        <v>57</v>
+      </c>
+      <c r="W9" t="s">
+        <v>169</v>
+      </c>
+      <c r="X9" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y9" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z9" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA9" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB9" t="s">
         <v>61</v>
-      </c>
-      <c r="N9" t="s">
-        <v>157</v>
-      </c>
-      <c r="O9" t="s">
-        <v>158</v>
-      </c>
-      <c r="P9" t="s">
-        <v>159</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>65</v>
-      </c>
-      <c r="R9" t="s">
-        <v>66</v>
-      </c>
-      <c r="S9" t="s">
-        <v>46</v>
-      </c>
-      <c r="T9" t="s">
-        <v>47</v>
-      </c>
-      <c r="U9" t="s">
-        <v>67</v>
-      </c>
-      <c r="V9" t="s">
-        <v>49</v>
-      </c>
-      <c r="W9" t="s">
-        <v>160</v>
-      </c>
-      <c r="X9" t="s">
-        <v>51</v>
-      </c>
-      <c r="Y9" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z9" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA9" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB9" t="s">
-        <v>53</v>
       </c>
       <c r="AC9">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:29" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>161</v>
+        <v>170</v>
       </c>
       <c r="C10" t="s">
+        <v>79</v>
+      </c>
+      <c r="D10" t="s">
+        <v>171</v>
+      </c>
+      <c r="E10" t="s">
+        <v>40</v>
+      </c>
+      <c r="F10" t="s">
+        <v>41</v>
+      </c>
+      <c r="G10" t="s">
+        <v>172</v>
+      </c>
+      <c r="H10" t="s">
+        <v>173</v>
+      </c>
+      <c r="I10" t="s">
+        <v>174</v>
+      </c>
+      <c r="J10" t="s">
+        <v>45</v>
+      </c>
+      <c r="K10" t="s">
+        <v>175</v>
+      </c>
+      <c r="L10" t="s">
+        <v>176</v>
+      </c>
+      <c r="M10" t="s">
+        <v>86</v>
+      </c>
+      <c r="N10" t="s">
+        <v>177</v>
+      </c>
+      <c r="O10" t="s">
         <v>71</v>
       </c>
-      <c r="D10" t="s">
-        <v>162</v>
-      </c>
-      <c r="E10" t="s">
-        <v>32</v>
-      </c>
-      <c r="F10" t="s">
-        <v>33</v>
-      </c>
-      <c r="G10" t="s">
-        <v>163</v>
-      </c>
-      <c r="H10" t="s">
-        <v>164</v>
-      </c>
-      <c r="I10" t="s">
-        <v>165</v>
-      </c>
-      <c r="J10" t="s">
-        <v>37</v>
-      </c>
-      <c r="K10" t="s">
-        <v>166</v>
-      </c>
-      <c r="L10" t="s">
-        <v>167</v>
-      </c>
-      <c r="M10" t="s">
-        <v>78</v>
-      </c>
-      <c r="N10" t="s">
-        <v>168</v>
-      </c>
-      <c r="O10" t="s">
-        <v>63</v>
-      </c>
       <c r="P10" t="s">
-        <v>169</v>
+        <v>178</v>
       </c>
       <c r="Q10" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="R10" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="S10" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T10" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U10" t="s">
-        <v>85</v>
+        <v>93</v>
       </c>
       <c r="V10" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="W10" t="s">
-        <v>170</v>
+        <v>179</v>
       </c>
       <c r="X10" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y10" t="s">
-        <v>88</v>
+        <v>96</v>
       </c>
       <c r="Z10" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA10" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB10" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC10">
         <v>0</v>
+      </c>
+      <c r="AD10" t="s">
+        <v>180</v>
+      </c>
+      <c r="AE10" t="s">
+        <v>86</v>
+      </c>
+      <c r="AF10" t="s">
+        <v>181</v>
+      </c>
+      <c r="AG10" t="s">
+        <v>71</v>
+      </c>
+      <c r="AH10" t="s">
+        <v>178</v>
+      </c>
+      <c r="AI10" t="s">
+        <v>90</v>
+      </c>
+      <c r="AJ10" t="s">
+        <v>91</v>
+      </c>
+      <c r="AK10" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="11" spans="1:29" x14ac:dyDescent="0.25">
@@ -1931,85 +2019,85 @@
         <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>171</v>
+        <v>182</v>
       </c>
       <c r="C11" t="s">
-        <v>30</v>
+        <v>38</v>
       </c>
       <c r="D11" t="s">
-        <v>172</v>
+        <v>183</v>
       </c>
       <c r="E11" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F11" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G11" t="s">
-        <v>173</v>
+        <v>184</v>
       </c>
       <c r="H11" t="s">
-        <v>174</v>
+        <v>185</v>
       </c>
       <c r="I11" t="s">
-        <v>175</v>
+        <v>186</v>
       </c>
       <c r="J11" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K11" t="s">
-        <v>176</v>
+        <v>187</v>
       </c>
       <c r="L11" t="s">
-        <v>177</v>
+        <v>188</v>
       </c>
       <c r="M11" t="s">
-        <v>96</v>
+        <v>104</v>
       </c>
       <c r="N11" t="s">
-        <v>178</v>
+        <v>189</v>
       </c>
       <c r="O11" t="s">
-        <v>42</v>
+        <v>50</v>
       </c>
       <c r="P11" t="s">
-        <v>179</v>
+        <v>190</v>
       </c>
       <c r="Q11" t="s">
-        <v>83</v>
+        <v>91</v>
       </c>
       <c r="R11" t="s">
-        <v>100</v>
+        <v>108</v>
       </c>
       <c r="S11" t="s">
-        <v>46</v>
+        <v>54</v>
       </c>
       <c r="T11" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U11" t="s">
-        <v>102</v>
+        <v>110</v>
       </c>
       <c r="V11" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W11" t="s">
-        <v>180</v>
+        <v>191</v>
       </c>
       <c r="X11" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y11" t="s">
-        <v>104</v>
+        <v>112</v>
       </c>
       <c r="Z11" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA11" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB11" t="s">
-        <v>181</v>
+        <v>192</v>
       </c>
       <c r="AC11">
         <v>0</v>
@@ -2020,85 +2108,85 @@
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>182</v>
+        <v>193</v>
       </c>
       <c r="C12" t="s">
-        <v>106</v>
+        <v>114</v>
       </c>
       <c r="D12" t="s">
-        <v>183</v>
+        <v>194</v>
       </c>
       <c r="E12" t="s">
-        <v>32</v>
+        <v>40</v>
       </c>
       <c r="F12" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="G12" t="s">
-        <v>184</v>
+        <v>195</v>
       </c>
       <c r="H12" t="s">
-        <v>185</v>
+        <v>196</v>
       </c>
       <c r="I12" t="s">
-        <v>186</v>
+        <v>197</v>
       </c>
       <c r="J12" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K12" t="s">
-        <v>187</v>
+        <v>198</v>
       </c>
       <c r="L12" t="s">
-        <v>188</v>
+        <v>199</v>
       </c>
       <c r="M12" t="s">
-        <v>113</v>
+        <v>121</v>
       </c>
       <c r="N12" t="s">
-        <v>189</v>
+        <v>200</v>
       </c>
       <c r="O12" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="P12" t="s">
-        <v>190</v>
+        <v>201</v>
       </c>
       <c r="Q12" t="s">
-        <v>117</v>
+        <v>125</v>
       </c>
       <c r="R12" t="s">
-        <v>44</v>
+        <v>52</v>
       </c>
       <c r="S12" t="s">
-        <v>191</v>
+        <v>202</v>
       </c>
       <c r="T12" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="U12" t="s">
-        <v>118</v>
+        <v>126</v>
       </c>
       <c r="V12" t="s">
-        <v>49</v>
+        <v>57</v>
       </c>
       <c r="W12" t="s">
-        <v>192</v>
+        <v>203</v>
       </c>
       <c r="X12" t="s">
-        <v>51</v>
+        <v>59</v>
       </c>
       <c r="Y12" t="s">
-        <v>121</v>
+        <v>129</v>
       </c>
       <c r="Z12" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AA12" t="s">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="AB12" t="s">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="AC12">
         <v>0</v>
@@ -2109,85 +2197,85 @@
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>193</v>
+        <v>204</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>79</v>
       </c>
       <c r="D13" t="s">
-        <v>194</v>
+        <v>205</v>
       </c>
       <c r="E13" t="s">
-        <v>195</v>
+        <v>206</v>
       </c>
       <c r="F13" t="s">
-        <v>196</v>
+        <v>207</v>
       </c>
       <c r="G13" t="s">
-        <v>197</v>
+        <v>208</v>
       </c>
       <c r="H13" t="s">
-        <v>198</v>
+        <v>209</v>
       </c>
       <c r="I13" t="s">
-        <v>199</v>
+        <v>210</v>
       </c>
       <c r="J13" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="K13" t="s">
-        <v>200</v>
+        <v>211</v>
       </c>
       <c r="L13" t="s">
-        <v>201</v>
+        <v>212</v>
       </c>
       <c r="M13" t="s">
+        <v>69</v>
+      </c>
+      <c r="N13" t="s">
+        <v>213</v>
+      </c>
+      <c r="O13" t="s">
+        <v>106</v>
+      </c>
+      <c r="P13" t="s">
+        <v>214</v>
+      </c>
+      <c r="Q13" t="s">
+        <v>73</v>
+      </c>
+      <c r="R13" t="s">
+        <v>74</v>
+      </c>
+      <c r="S13" t="s">
+        <v>54</v>
+      </c>
+      <c r="T13" t="s">
+        <v>55</v>
+      </c>
+      <c r="U13" t="s">
+        <v>75</v>
+      </c>
+      <c r="V13" t="s">
+        <v>94</v>
+      </c>
+      <c r="W13" t="s">
+        <v>215</v>
+      </c>
+      <c r="X13" t="s">
+        <v>59</v>
+      </c>
+      <c r="Y13" t="s">
+        <v>77</v>
+      </c>
+      <c r="Z13" t="s">
+        <v>41</v>
+      </c>
+      <c r="AA13" t="s">
+        <v>41</v>
+      </c>
+      <c r="AB13" t="s">
         <v>61</v>
-      </c>
-      <c r="N13" t="s">
-        <v>202</v>
-      </c>
-      <c r="O13" t="s">
-        <v>98</v>
-      </c>
-      <c r="P13" t="s">
-        <v>203</v>
-      </c>
-      <c r="Q13" t="s">
-        <v>65</v>
-      </c>
-      <c r="R13" t="s">
-        <v>66</v>
-      </c>
-      <c r="S13" t="s">
-        <v>46</v>
-      </c>
-      <c r="T13" t="s">
-        <v>47</v>
-      </c>
-      <c r="U13" t="s">
-        <v>67</v>
-      </c>
-      <c r="V13" t="s">
-        <v>86</v>
-      </c>
-      <c r="W13" t="s">
-        <v>204</v>
-      </c>
-      <c r="X13" t="s">
-        <v>51</v>
-      </c>
-      <c r="Y13" t="s">
-        <v>69</v>
-      </c>
-      <c r="Z13" t="s">
-        <v>33</v>
-      </c>
-      <c r="AA13" t="s">
-        <v>33</v>
-      </c>
-      <c r="AB13" t="s">
-        <v>53</v>
       </c>
       <c r="AC13">
         <v>0</v>

</xml_diff>